<commit_message>
Updated some UI, added live server setup details
</commit_message>
<xml_diff>
--- a/frontend/public/templates/DailyReportTemplate.xlsx
+++ b/frontend/public/templates/DailyReportTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\productivity_report\frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF4EEA57-F3FB-4A7B-BCDB-8A81BF9C9858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CD83758-B1F1-4F91-A86D-A7024886BB51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-4740" windowWidth="29040" windowHeight="15720" xr2:uid="{B7467352-BE85-4F3F-BF29-5BEED4CA8646}"/>
   </bookViews>
@@ -130,7 +130,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -492,6 +510,12 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A2:G1048576">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$C2="Holiday"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>